<commit_message>
Human golden-50 labels (Bailey), logged corrections, import normalization
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evals/golden/golden_50_label_sheet.xlsx
+++ b/evals/golden/golden_50_label_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fe8181242c3803c0/Documents/Academics/Year 2/Agentic AI/13OCT2026_Capstone Project/evals/golden/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_AA472F57724F4A6397D4BC430FD4FC93FFAEE010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25B5928D-3BFF-44C2-8DD7-854131E5D712}"/>
+  <xr:revisionPtr revIDLastSave="512" documentId="11_AA472F57724F4A6397D4BC430FD4FC93FFAEE010" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18F01D1A-7E61-4078-85E8-86AE18AF33EA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="295">
   <si>
     <t>HOW TO LABEL (label the text only; ignore stars; you are the human reference)</t>
   </si>
@@ -737,15 +737,15 @@
     <t>other_specific</t>
   </si>
   <si>
-    <t>"Staff must be full of mentally ill kool-aid heads", "Spotify is doing all they can to protect pedophiles"</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
     <t>"Great app"</t>
   </si>
   <si>
+    <t>"Excellent"</t>
+  </si>
+  <si>
     <t>"an amazing experience"</t>
   </si>
   <si>
@@ -753,6 +753,162 @@
   </si>
   <si>
     <t>"loved it"</t>
+  </si>
+  <si>
+    <t>"hate this application"</t>
+  </si>
+  <si>
+    <t>"good"</t>
+  </si>
+  <si>
+    <t>"Great"</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>May not be speaking about Spotify Premium, and Duolingo instead</t>
+  </si>
+  <si>
+    <t>two experiencesone positive with Support and one negative with the crashing issue in the same comment, changing the meaning</t>
+  </si>
+  <si>
+    <t>"app is bad work"</t>
+  </si>
+  <si>
+    <t>"Super"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">that is not the normal functionality/intent of using Spotify. Not sure what this guy is getting at. </t>
+  </si>
+  <si>
+    <t>In a different language</t>
+  </si>
+  <si>
+    <t>"We are boycotting"</t>
+  </si>
+  <si>
+    <t>"🙄"</t>
+  </si>
+  <si>
+    <t>"Awesomeness"</t>
+  </si>
+  <si>
+    <t>"unconditional love"</t>
+  </si>
+  <si>
+    <t>Unclear meaning</t>
+  </si>
+  <si>
+    <t>several complaints rolled into one comment</t>
+  </si>
+  <si>
+    <t>"everything basic features is premium"</t>
+  </si>
+  <si>
+    <t>"Good"</t>
+  </si>
+  <si>
+    <t>"Good app!"</t>
+  </si>
+  <si>
+    <t>"I hate this app"</t>
+  </si>
+  <si>
+    <t>referred to Sweden boycott</t>
+  </si>
+  <si>
+    <t>I really loved spotify but this making me to rate it 1 star"</t>
+  </si>
+  <si>
+    <t>Ads</t>
+  </si>
+  <si>
+    <t>off topic</t>
+  </si>
+  <si>
+    <t>"bro I can't be like"</t>
+  </si>
+  <si>
+    <t>Not sure what the phrase is trying to communicate</t>
+  </si>
+  <si>
+    <t>"Phenomenal"</t>
+  </si>
+  <si>
+    <t>general praise</t>
+  </si>
+  <si>
+    <t>"Worst app"</t>
+  </si>
+  <si>
+    <t>"very good"</t>
+  </si>
+  <si>
+    <t>"paying for subscribing but unable to play in offline mode really"</t>
+  </si>
+  <si>
+    <t>"best app ever"</t>
+  </si>
+  <si>
+    <t>"loving the experience"</t>
+  </si>
+  <si>
+    <t>"this update very bad for everyone."</t>
+  </si>
+  <si>
+    <t>"Staff must be full of mentally ill kool-aid heads"; "Spotify is doing all they can to protect pedophiles"</t>
+  </si>
+  <si>
+    <t>"hate this application"; "🤮"</t>
+  </si>
+  <si>
+    <t>"awesome"; "very diverse"</t>
+  </si>
+  <si>
+    <t>"Duo Premium"; "No ads at all!"</t>
+  </si>
+  <si>
+    <t>"plays a little bit then it stops"; "fix this issue"</t>
+  </si>
+  <si>
+    <t>"it keeps crashing every time"; "Nothing seems to work unfortunately"</t>
+  </si>
+  <si>
+    <t>"I like it"; "I hate it when"</t>
+  </si>
+  <si>
+    <t>"I LOVE that"; "Awesome"</t>
+  </si>
+  <si>
+    <t>"I absolutely love Spotify"; "Great Job"</t>
+  </si>
+  <si>
+    <t>"Very poor updates"; "It is affecting the spotify quality"</t>
+  </si>
+  <si>
+    <t>"new update suck"; "no wonder if you guys loose ratings and users"</t>
+  </si>
+  <si>
+    <t>"This is dangerous"; "stop this BS"</t>
+  </si>
+  <si>
+    <t>"nice app"; "Very less advertising"</t>
+  </si>
+  <si>
+    <t>"pathetic update"; "Lyrics not getting loaded"</t>
+  </si>
+  <si>
+    <t>"would definitely deserve 5 stars if"; "The only thing Spotify lacks"</t>
+  </si>
+  <si>
+    <t>"one star"; "annoying"</t>
+  </si>
+  <si>
+    <t>"worst app ever"; "too many ads"</t>
+  </si>
+  <si>
+    <t>"too expensive"; "free version is unusable"</t>
   </si>
 </sst>
 </file>
@@ -1550,10 +1706,10 @@
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>237</v>
+        <v>277</v>
       </c>
       <c r="J2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K2" t="s">
         <v>191</v>
@@ -1573,7 +1729,7 @@
         <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="E3" t="s">
         <v>233</v>
@@ -1588,10 +1744,10 @@
         <v>201</v>
       </c>
       <c r="I3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K3" t="s">
         <v>191</v>
@@ -1629,7 +1785,7 @@
         <v>240</v>
       </c>
       <c r="J4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K4" t="s">
         <v>191</v>
@@ -1704,6 +1860,15 @@
       <c r="I6" t="s">
         <v>242</v>
       </c>
+      <c r="J6" t="s">
+        <v>237</v>
+      </c>
+      <c r="K6" t="s">
+        <v>191</v>
+      </c>
+      <c r="L6" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7">
@@ -1715,6 +1880,33 @@
       <c r="C7" s="3" t="s">
         <v>92</v>
       </c>
+      <c r="D7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F7" t="s">
+        <v>188</v>
+      </c>
+      <c r="G7" t="s">
+        <v>189</v>
+      </c>
+      <c r="H7" t="s">
+        <v>184</v>
+      </c>
+      <c r="I7" t="s">
+        <v>278</v>
+      </c>
+      <c r="J7" t="s">
+        <v>237</v>
+      </c>
+      <c r="K7" t="s">
+        <v>191</v>
+      </c>
+      <c r="L7" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8">
@@ -1726,6 +1918,33 @@
       <c r="C8" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="D8" t="s">
+        <v>210</v>
+      </c>
+      <c r="E8" t="s">
+        <v>233</v>
+      </c>
+      <c r="F8" t="s">
+        <v>199</v>
+      </c>
+      <c r="G8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I8" t="s">
+        <v>239</v>
+      </c>
+      <c r="J8" t="s">
+        <v>237</v>
+      </c>
+      <c r="K8" t="s">
+        <v>191</v>
+      </c>
+      <c r="L8" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9">
@@ -1737,6 +1956,33 @@
       <c r="C9" s="3" t="s">
         <v>96</v>
       </c>
+      <c r="D9" t="s">
+        <v>210</v>
+      </c>
+      <c r="E9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F9" t="s">
+        <v>199</v>
+      </c>
+      <c r="G9" t="s">
+        <v>183</v>
+      </c>
+      <c r="H9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I9" t="s">
+        <v>244</v>
+      </c>
+      <c r="J9" t="s">
+        <v>237</v>
+      </c>
+      <c r="K9" t="s">
+        <v>191</v>
+      </c>
+      <c r="L9" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10">
@@ -1748,6 +1994,33 @@
       <c r="C10" s="3" t="s">
         <v>98</v>
       </c>
+      <c r="D10" t="s">
+        <v>210</v>
+      </c>
+      <c r="E10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F10" t="s">
+        <v>199</v>
+      </c>
+      <c r="G10" t="s">
+        <v>183</v>
+      </c>
+      <c r="H10" t="s">
+        <v>183</v>
+      </c>
+      <c r="I10" t="s">
+        <v>279</v>
+      </c>
+      <c r="J10" t="s">
+        <v>237</v>
+      </c>
+      <c r="K10" t="s">
+        <v>191</v>
+      </c>
+      <c r="L10" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11">
@@ -1759,6 +2032,36 @@
       <c r="C11" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="D11" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F11" t="s">
+        <v>204</v>
+      </c>
+      <c r="G11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H11" t="s">
+        <v>196</v>
+      </c>
+      <c r="I11" t="s">
+        <v>280</v>
+      </c>
+      <c r="J11" t="s">
+        <v>246</v>
+      </c>
+      <c r="K11" t="s">
+        <v>185</v>
+      </c>
+      <c r="L11" t="s">
+        <v>185</v>
+      </c>
+      <c r="P11" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A12">
@@ -1770,6 +2073,33 @@
       <c r="C12" s="3" t="s">
         <v>102</v>
       </c>
+      <c r="D12" t="s">
+        <v>192</v>
+      </c>
+      <c r="E12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F12" t="s">
+        <v>188</v>
+      </c>
+      <c r="G12" t="s">
+        <v>195</v>
+      </c>
+      <c r="H12" t="s">
+        <v>190</v>
+      </c>
+      <c r="I12" t="s">
+        <v>281</v>
+      </c>
+      <c r="J12" t="s">
+        <v>237</v>
+      </c>
+      <c r="K12" t="s">
+        <v>191</v>
+      </c>
+      <c r="L12" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="13" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13">
@@ -1781,6 +2111,45 @@
       <c r="C13" s="3" t="s">
         <v>104</v>
       </c>
+      <c r="D13" t="s">
+        <v>192</v>
+      </c>
+      <c r="E13" t="s">
+        <v>214</v>
+      </c>
+      <c r="F13" t="s">
+        <v>188</v>
+      </c>
+      <c r="G13" t="s">
+        <v>200</v>
+      </c>
+      <c r="H13" t="s">
+        <v>190</v>
+      </c>
+      <c r="I13" t="s">
+        <v>282</v>
+      </c>
+      <c r="J13" t="s">
+        <v>237</v>
+      </c>
+      <c r="K13" t="s">
+        <v>185</v>
+      </c>
+      <c r="L13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M13" t="s">
+        <v>208</v>
+      </c>
+      <c r="N13" t="s">
+        <v>199</v>
+      </c>
+      <c r="O13" t="s">
+        <v>183</v>
+      </c>
+      <c r="P13" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14">
@@ -1792,6 +2161,33 @@
       <c r="C14" s="3" t="s">
         <v>106</v>
       </c>
+      <c r="D14" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" t="s">
+        <v>234</v>
+      </c>
+      <c r="F14" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" t="s">
+        <v>189</v>
+      </c>
+      <c r="H14" t="s">
+        <v>184</v>
+      </c>
+      <c r="I14" t="s">
+        <v>249</v>
+      </c>
+      <c r="J14" t="s">
+        <v>237</v>
+      </c>
+      <c r="K14" t="s">
+        <v>191</v>
+      </c>
+      <c r="L14" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15">
@@ -1803,6 +2199,33 @@
       <c r="C15" s="3" t="s">
         <v>108</v>
       </c>
+      <c r="D15" t="s">
+        <v>210</v>
+      </c>
+      <c r="E15" t="s">
+        <v>233</v>
+      </c>
+      <c r="F15" t="s">
+        <v>199</v>
+      </c>
+      <c r="G15" t="s">
+        <v>183</v>
+      </c>
+      <c r="H15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I15" t="s">
+        <v>245</v>
+      </c>
+      <c r="J15" t="s">
+        <v>237</v>
+      </c>
+      <c r="K15" t="s">
+        <v>191</v>
+      </c>
+      <c r="L15" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16">
@@ -1814,8 +2237,35 @@
       <c r="C16" s="3" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16" t="s">
+        <v>210</v>
+      </c>
+      <c r="E16" t="s">
+        <v>233</v>
+      </c>
+      <c r="F16" t="s">
+        <v>199</v>
+      </c>
+      <c r="G16" t="s">
+        <v>183</v>
+      </c>
+      <c r="H16" t="s">
+        <v>183</v>
+      </c>
+      <c r="I16" t="s">
+        <v>250</v>
+      </c>
+      <c r="J16" t="s">
+        <v>237</v>
+      </c>
+      <c r="K16" t="s">
+        <v>191</v>
+      </c>
+      <c r="L16" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1825,8 +2275,47 @@
       <c r="C17" s="3" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17" t="s">
+        <v>186</v>
+      </c>
+      <c r="E17" t="s">
+        <v>236</v>
+      </c>
+      <c r="F17" t="s">
+        <v>204</v>
+      </c>
+      <c r="G17" t="s">
+        <v>189</v>
+      </c>
+      <c r="H17" t="s">
+        <v>190</v>
+      </c>
+      <c r="I17" t="s">
+        <v>283</v>
+      </c>
+      <c r="J17" t="s">
+        <v>237</v>
+      </c>
+      <c r="K17" t="s">
+        <v>185</v>
+      </c>
+      <c r="L17" t="s">
+        <v>185</v>
+      </c>
+      <c r="M17" t="s">
+        <v>180</v>
+      </c>
+      <c r="N17" t="s">
+        <v>188</v>
+      </c>
+      <c r="O17" t="s">
+        <v>183</v>
+      </c>
+      <c r="P17" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1836,8 +2325,35 @@
       <c r="C18" s="3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18" t="s">
+        <v>210</v>
+      </c>
+      <c r="E18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G18" t="s">
+        <v>183</v>
+      </c>
+      <c r="H18" t="s">
+        <v>196</v>
+      </c>
+      <c r="J18" t="s">
+        <v>237</v>
+      </c>
+      <c r="K18" t="s">
+        <v>185</v>
+      </c>
+      <c r="L18" t="s">
+        <v>185</v>
+      </c>
+      <c r="P18" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1847,8 +2363,32 @@
       <c r="C19" s="3" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>236</v>
+      </c>
+      <c r="F19" t="s">
+        <v>204</v>
+      </c>
+      <c r="G19" t="s">
+        <v>183</v>
+      </c>
+      <c r="H19" t="s">
+        <v>196</v>
+      </c>
+      <c r="K19" t="s">
+        <v>185</v>
+      </c>
+      <c r="L19" t="s">
+        <v>185</v>
+      </c>
+      <c r="P19" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1858,8 +2398,32 @@
       <c r="C20" s="3" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20" t="s">
+        <v>210</v>
+      </c>
+      <c r="E20" t="s">
+        <v>236</v>
+      </c>
+      <c r="F20" t="s">
+        <v>204</v>
+      </c>
+      <c r="G20" t="s">
+        <v>183</v>
+      </c>
+      <c r="H20" t="s">
+        <v>196</v>
+      </c>
+      <c r="K20" t="s">
+        <v>185</v>
+      </c>
+      <c r="L20" t="s">
+        <v>185</v>
+      </c>
+      <c r="P20" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1869,8 +2433,35 @@
       <c r="C21" s="3" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D21" t="s">
+        <v>210</v>
+      </c>
+      <c r="E21" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" t="s">
+        <v>188</v>
+      </c>
+      <c r="G21" t="s">
+        <v>189</v>
+      </c>
+      <c r="H21" t="s">
+        <v>184</v>
+      </c>
+      <c r="I21" t="s">
+        <v>243</v>
+      </c>
+      <c r="J21" t="s">
+        <v>237</v>
+      </c>
+      <c r="K21" t="s">
+        <v>191</v>
+      </c>
+      <c r="L21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1880,8 +2471,35 @@
       <c r="C22" s="3" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D22" t="s">
+        <v>210</v>
+      </c>
+      <c r="E22" t="s">
+        <v>235</v>
+      </c>
+      <c r="F22" t="s">
+        <v>204</v>
+      </c>
+      <c r="G22" t="s">
+        <v>189</v>
+      </c>
+      <c r="H22" t="s">
+        <v>184</v>
+      </c>
+      <c r="I22" t="s">
+        <v>253</v>
+      </c>
+      <c r="J22" t="s">
+        <v>237</v>
+      </c>
+      <c r="K22" t="s">
+        <v>191</v>
+      </c>
+      <c r="L22" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1891,8 +2509,35 @@
       <c r="C23" s="3" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23" t="s">
+        <v>186</v>
+      </c>
+      <c r="E23" t="s">
+        <v>209</v>
+      </c>
+      <c r="F23" t="s">
+        <v>199</v>
+      </c>
+      <c r="G23" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" t="s">
+        <v>183</v>
+      </c>
+      <c r="I23" t="s">
+        <v>284</v>
+      </c>
+      <c r="J23" t="s">
+        <v>237</v>
+      </c>
+      <c r="K23" t="s">
+        <v>191</v>
+      </c>
+      <c r="L23" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1902,8 +2547,35 @@
       <c r="C24" s="3" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24" t="s">
+        <v>210</v>
+      </c>
+      <c r="E24" t="s">
+        <v>233</v>
+      </c>
+      <c r="F24" t="s">
+        <v>199</v>
+      </c>
+      <c r="G24" t="s">
+        <v>183</v>
+      </c>
+      <c r="H24" t="s">
+        <v>183</v>
+      </c>
+      <c r="I24" t="s">
+        <v>285</v>
+      </c>
+      <c r="J24" t="s">
+        <v>237</v>
+      </c>
+      <c r="K24" t="s">
+        <v>191</v>
+      </c>
+      <c r="L24" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1913,8 +2585,38 @@
       <c r="C25" s="3" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D25" t="s">
+        <v>210</v>
+      </c>
+      <c r="E25" t="s">
+        <v>234</v>
+      </c>
+      <c r="F25" t="s">
+        <v>204</v>
+      </c>
+      <c r="G25" t="s">
+        <v>189</v>
+      </c>
+      <c r="H25" t="s">
+        <v>190</v>
+      </c>
+      <c r="I25" t="s">
+        <v>254</v>
+      </c>
+      <c r="J25" t="s">
+        <v>237</v>
+      </c>
+      <c r="K25" t="s">
+        <v>185</v>
+      </c>
+      <c r="L25" t="s">
+        <v>185</v>
+      </c>
+      <c r="P25" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1924,8 +2626,35 @@
       <c r="C26" s="3" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26" t="s">
+        <v>192</v>
+      </c>
+      <c r="E26" t="s">
+        <v>212</v>
+      </c>
+      <c r="F26" t="s">
+        <v>188</v>
+      </c>
+      <c r="G26" t="s">
+        <v>195</v>
+      </c>
+      <c r="H26" t="s">
+        <v>184</v>
+      </c>
+      <c r="I26" t="s">
+        <v>286</v>
+      </c>
+      <c r="J26" t="s">
+        <v>237</v>
+      </c>
+      <c r="K26" t="s">
+        <v>191</v>
+      </c>
+      <c r="L26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1935,8 +2664,35 @@
       <c r="C27" s="3" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D27" t="s">
+        <v>210</v>
+      </c>
+      <c r="E27" t="s">
+        <v>233</v>
+      </c>
+      <c r="F27" t="s">
+        <v>199</v>
+      </c>
+      <c r="G27" t="s">
+        <v>183</v>
+      </c>
+      <c r="H27" t="s">
+        <v>183</v>
+      </c>
+      <c r="I27" t="s">
+        <v>255</v>
+      </c>
+      <c r="J27" t="s">
+        <v>237</v>
+      </c>
+      <c r="K27" t="s">
+        <v>191</v>
+      </c>
+      <c r="L27" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1946,8 +2702,35 @@
       <c r="C28" s="3" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D28" t="s">
+        <v>210</v>
+      </c>
+      <c r="E28" t="s">
+        <v>233</v>
+      </c>
+      <c r="F28" t="s">
+        <v>204</v>
+      </c>
+      <c r="G28" t="s">
+        <v>183</v>
+      </c>
+      <c r="H28" t="s">
+        <v>196</v>
+      </c>
+      <c r="J28" t="s">
+        <v>237</v>
+      </c>
+      <c r="K28" t="s">
+        <v>185</v>
+      </c>
+      <c r="L28" t="s">
+        <v>185</v>
+      </c>
+      <c r="P28" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1957,8 +2740,32 @@
       <c r="C29" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="D29" t="s">
+        <v>210</v>
+      </c>
+      <c r="E29" t="s">
+        <v>233</v>
+      </c>
+      <c r="F29" t="s">
+        <v>204</v>
+      </c>
+      <c r="G29" t="s">
+        <v>183</v>
+      </c>
+      <c r="H29" t="s">
+        <v>196</v>
+      </c>
+      <c r="I29" t="s">
+        <v>256</v>
+      </c>
+      <c r="J29" t="s">
+        <v>237</v>
+      </c>
+      <c r="P29" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1968,8 +2775,38 @@
       <c r="C30" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D30" t="s">
+        <v>186</v>
+      </c>
+      <c r="E30" t="s">
+        <v>234</v>
+      </c>
+      <c r="F30" t="s">
+        <v>182</v>
+      </c>
+      <c r="G30" t="s">
+        <v>205</v>
+      </c>
+      <c r="H30" t="s">
+        <v>184</v>
+      </c>
+      <c r="I30" t="s">
+        <v>287</v>
+      </c>
+      <c r="J30" t="s">
+        <v>246</v>
+      </c>
+      <c r="K30" t="s">
+        <v>185</v>
+      </c>
+      <c r="L30" t="s">
+        <v>185</v>
+      </c>
+      <c r="P30" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1979,8 +2816,35 @@
       <c r="C31" s="3" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D31" t="s">
+        <v>206</v>
+      </c>
+      <c r="E31" t="s">
+        <v>227</v>
+      </c>
+      <c r="F31" t="s">
+        <v>188</v>
+      </c>
+      <c r="G31" t="s">
+        <v>195</v>
+      </c>
+      <c r="H31" t="s">
+        <v>184</v>
+      </c>
+      <c r="I31" t="s">
+        <v>259</v>
+      </c>
+      <c r="J31" t="s">
+        <v>246</v>
+      </c>
+      <c r="K31" t="s">
+        <v>191</v>
+      </c>
+      <c r="L31" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1990,8 +2854,38 @@
       <c r="C32" s="3" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="D32" t="s">
+        <v>210</v>
+      </c>
+      <c r="E32" t="s">
+        <v>235</v>
+      </c>
+      <c r="F32" t="s">
+        <v>188</v>
+      </c>
+      <c r="G32" t="s">
+        <v>189</v>
+      </c>
+      <c r="H32" t="s">
+        <v>184</v>
+      </c>
+      <c r="I32" t="s">
+        <v>262</v>
+      </c>
+      <c r="J32" t="s">
+        <v>237</v>
+      </c>
+      <c r="K32" t="s">
+        <v>191</v>
+      </c>
+      <c r="L32" t="s">
+        <v>191</v>
+      </c>
+      <c r="P32" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="58" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2001,8 +2895,35 @@
       <c r="C33" s="3" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="D33" t="s">
+        <v>186</v>
+      </c>
+      <c r="E33" t="s">
+        <v>214</v>
+      </c>
+      <c r="F33" t="s">
+        <v>188</v>
+      </c>
+      <c r="G33" t="s">
+        <v>195</v>
+      </c>
+      <c r="H33" t="s">
+        <v>184</v>
+      </c>
+      <c r="I33" t="s">
+        <v>264</v>
+      </c>
+      <c r="J33" t="s">
+        <v>237</v>
+      </c>
+      <c r="K33" t="s">
+        <v>191</v>
+      </c>
+      <c r="L33" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2012,8 +2933,35 @@
       <c r="C34" s="3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D34" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" t="s">
+        <v>203</v>
+      </c>
+      <c r="F34" t="s">
+        <v>182</v>
+      </c>
+      <c r="G34" t="s">
+        <v>195</v>
+      </c>
+      <c r="H34" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" t="s">
+        <v>288</v>
+      </c>
+      <c r="J34" t="s">
+        <v>265</v>
+      </c>
+      <c r="K34" t="s">
+        <v>191</v>
+      </c>
+      <c r="L34" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2023,8 +2971,38 @@
       <c r="C35" s="3" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D35" t="s">
+        <v>210</v>
+      </c>
+      <c r="E35" t="s">
+        <v>266</v>
+      </c>
+      <c r="F35" t="s">
+        <v>204</v>
+      </c>
+      <c r="G35" t="s">
+        <v>183</v>
+      </c>
+      <c r="H35" t="s">
+        <v>196</v>
+      </c>
+      <c r="I35" t="s">
+        <v>267</v>
+      </c>
+      <c r="J35" t="s">
+        <v>237</v>
+      </c>
+      <c r="K35" t="s">
+        <v>185</v>
+      </c>
+      <c r="L35" t="s">
+        <v>185</v>
+      </c>
+      <c r="P35" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2034,8 +3012,35 @@
       <c r="C36" s="3" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E36" t="s">
+        <v>233</v>
+      </c>
+      <c r="F36" t="s">
+        <v>199</v>
+      </c>
+      <c r="G36" t="s">
+        <v>183</v>
+      </c>
+      <c r="H36" t="s">
+        <v>183</v>
+      </c>
+      <c r="I36" t="s">
+        <v>260</v>
+      </c>
+      <c r="J36" t="s">
+        <v>237</v>
+      </c>
+      <c r="K36" t="s">
+        <v>191</v>
+      </c>
+      <c r="L36" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2045,8 +3050,35 @@
       <c r="C37" s="3" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D37" t="s">
+        <v>210</v>
+      </c>
+      <c r="E37" t="s">
+        <v>233</v>
+      </c>
+      <c r="F37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G37" t="s">
+        <v>183</v>
+      </c>
+      <c r="H37" t="s">
+        <v>183</v>
+      </c>
+      <c r="I37" t="s">
+        <v>261</v>
+      </c>
+      <c r="J37" t="s">
+        <v>237</v>
+      </c>
+      <c r="K37" t="s">
+        <v>191</v>
+      </c>
+      <c r="L37" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2056,8 +3088,35 @@
       <c r="C38" s="3" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D38" t="s">
+        <v>186</v>
+      </c>
+      <c r="E38" t="s">
+        <v>203</v>
+      </c>
+      <c r="F38" t="s">
+        <v>199</v>
+      </c>
+      <c r="G38" t="s">
+        <v>183</v>
+      </c>
+      <c r="H38" t="s">
+        <v>183</v>
+      </c>
+      <c r="I38" t="s">
+        <v>289</v>
+      </c>
+      <c r="J38" t="s">
+        <v>265</v>
+      </c>
+      <c r="K38" t="s">
+        <v>191</v>
+      </c>
+      <c r="L38" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2067,8 +3126,35 @@
       <c r="C39" s="3" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D39" t="s">
+        <v>186</v>
+      </c>
+      <c r="E39" t="s">
+        <v>225</v>
+      </c>
+      <c r="F39" t="s">
+        <v>188</v>
+      </c>
+      <c r="G39" t="s">
+        <v>189</v>
+      </c>
+      <c r="H39" t="s">
+        <v>190</v>
+      </c>
+      <c r="I39" t="s">
+        <v>290</v>
+      </c>
+      <c r="J39" t="s">
+        <v>237</v>
+      </c>
+      <c r="K39" t="s">
+        <v>191</v>
+      </c>
+      <c r="L39" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2078,8 +3164,35 @@
       <c r="C40" s="3" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D40" t="s">
+        <v>210</v>
+      </c>
+      <c r="E40" t="s">
+        <v>233</v>
+      </c>
+      <c r="F40" t="s">
+        <v>199</v>
+      </c>
+      <c r="G40" t="s">
+        <v>183</v>
+      </c>
+      <c r="H40" t="s">
+        <v>183</v>
+      </c>
+      <c r="I40" t="s">
+        <v>269</v>
+      </c>
+      <c r="J40" t="s">
+        <v>237</v>
+      </c>
+      <c r="K40" t="s">
+        <v>191</v>
+      </c>
+      <c r="L40" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2089,8 +3202,35 @@
       <c r="C41" s="3" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="D41" t="s">
+        <v>210</v>
+      </c>
+      <c r="E41" t="s">
+        <v>270</v>
+      </c>
+      <c r="F41" t="s">
+        <v>199</v>
+      </c>
+      <c r="G41" t="s">
+        <v>183</v>
+      </c>
+      <c r="H41" t="s">
+        <v>183</v>
+      </c>
+      <c r="I41" t="s">
+        <v>260</v>
+      </c>
+      <c r="J41" t="s">
+        <v>237</v>
+      </c>
+      <c r="K41" t="s">
+        <v>191</v>
+      </c>
+      <c r="L41" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2100,8 +3240,35 @@
       <c r="C42" s="3" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D42" t="s">
+        <v>186</v>
+      </c>
+      <c r="E42" t="s">
+        <v>209</v>
+      </c>
+      <c r="F42" t="s">
+        <v>194</v>
+      </c>
+      <c r="G42" t="s">
+        <v>189</v>
+      </c>
+      <c r="H42" t="s">
+        <v>201</v>
+      </c>
+      <c r="I42" t="s">
+        <v>291</v>
+      </c>
+      <c r="J42" t="s">
+        <v>237</v>
+      </c>
+      <c r="K42" t="s">
+        <v>191</v>
+      </c>
+      <c r="L42" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2111,8 +3278,35 @@
       <c r="C43" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="D43" t="s">
+        <v>210</v>
+      </c>
+      <c r="E43" t="s">
+        <v>234</v>
+      </c>
+      <c r="F43" t="s">
+        <v>188</v>
+      </c>
+      <c r="G43" t="s">
+        <v>189</v>
+      </c>
+      <c r="H43" t="s">
+        <v>184</v>
+      </c>
+      <c r="I43" t="s">
+        <v>271</v>
+      </c>
+      <c r="J43" t="s">
+        <v>237</v>
+      </c>
+      <c r="K43" t="s">
+        <v>191</v>
+      </c>
+      <c r="L43" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2122,8 +3316,35 @@
       <c r="C44" s="3" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="D44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E44" t="s">
+        <v>211</v>
+      </c>
+      <c r="F44" t="s">
+        <v>188</v>
+      </c>
+      <c r="G44" t="s">
+        <v>205</v>
+      </c>
+      <c r="H44" t="s">
+        <v>184</v>
+      </c>
+      <c r="I44" t="s">
+        <v>292</v>
+      </c>
+      <c r="J44" t="s">
+        <v>237</v>
+      </c>
+      <c r="K44" t="s">
+        <v>191</v>
+      </c>
+      <c r="L44" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2133,8 +3354,35 @@
       <c r="C45" s="3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D45" t="s">
+        <v>186</v>
+      </c>
+      <c r="E45" t="s">
+        <v>209</v>
+      </c>
+      <c r="F45" t="s">
+        <v>199</v>
+      </c>
+      <c r="G45" t="s">
+        <v>183</v>
+      </c>
+      <c r="H45" t="s">
+        <v>183</v>
+      </c>
+      <c r="I45" t="s">
+        <v>272</v>
+      </c>
+      <c r="J45" t="s">
+        <v>237</v>
+      </c>
+      <c r="K45" t="s">
+        <v>191</v>
+      </c>
+      <c r="L45" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2144,8 +3392,35 @@
       <c r="C46" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D46" t="s">
+        <v>186</v>
+      </c>
+      <c r="E46" t="s">
+        <v>221</v>
+      </c>
+      <c r="F46" t="s">
+        <v>188</v>
+      </c>
+      <c r="G46" t="s">
+        <v>195</v>
+      </c>
+      <c r="H46" t="s">
+        <v>184</v>
+      </c>
+      <c r="I46" t="s">
+        <v>273</v>
+      </c>
+      <c r="J46" t="s">
+        <v>237</v>
+      </c>
+      <c r="K46" t="s">
+        <v>191</v>
+      </c>
+      <c r="L46" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2155,8 +3430,35 @@
       <c r="C47" s="3" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="D47" t="s">
+        <v>186</v>
+      </c>
+      <c r="E47" t="s">
+        <v>203</v>
+      </c>
+      <c r="F47" t="s">
+        <v>182</v>
+      </c>
+      <c r="G47" t="s">
+        <v>189</v>
+      </c>
+      <c r="H47" t="s">
+        <v>184</v>
+      </c>
+      <c r="I47" t="s">
+        <v>293</v>
+      </c>
+      <c r="J47" t="s">
+        <v>203</v>
+      </c>
+      <c r="K47" t="s">
+        <v>191</v>
+      </c>
+      <c r="L47" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2166,8 +3468,35 @@
       <c r="C48" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D48" t="s">
+        <v>206</v>
+      </c>
+      <c r="E48" t="s">
+        <v>228</v>
+      </c>
+      <c r="F48" t="s">
+        <v>188</v>
+      </c>
+      <c r="G48" t="s">
+        <v>195</v>
+      </c>
+      <c r="H48" t="s">
+        <v>184</v>
+      </c>
+      <c r="I48" t="s">
+        <v>294</v>
+      </c>
+      <c r="J48" t="s">
+        <v>237</v>
+      </c>
+      <c r="K48" t="s">
+        <v>191</v>
+      </c>
+      <c r="L48" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2177,8 +3506,35 @@
       <c r="C49" s="3" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49" t="s">
+        <v>186</v>
+      </c>
+      <c r="E49" t="s">
+        <v>234</v>
+      </c>
+      <c r="F49" t="s">
+        <v>188</v>
+      </c>
+      <c r="G49" t="s">
+        <v>189</v>
+      </c>
+      <c r="H49" t="s">
+        <v>184</v>
+      </c>
+      <c r="I49" t="s">
+        <v>276</v>
+      </c>
+      <c r="J49" t="s">
+        <v>237</v>
+      </c>
+      <c r="K49" t="s">
+        <v>191</v>
+      </c>
+      <c r="L49" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2188,8 +3544,35 @@
       <c r="C50" s="3" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D50" t="s">
+        <v>186</v>
+      </c>
+      <c r="E50" t="s">
+        <v>233</v>
+      </c>
+      <c r="F50" t="s">
+        <v>199</v>
+      </c>
+      <c r="G50" t="s">
+        <v>183</v>
+      </c>
+      <c r="H50" t="s">
+        <v>183</v>
+      </c>
+      <c r="I50" t="s">
+        <v>275</v>
+      </c>
+      <c r="J50" t="s">
+        <v>237</v>
+      </c>
+      <c r="K50" t="s">
+        <v>191</v>
+      </c>
+      <c r="L50" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2198,6 +3581,33 @@
       </c>
       <c r="C51" s="3" t="s">
         <v>179</v>
+      </c>
+      <c r="D51" t="s">
+        <v>210</v>
+      </c>
+      <c r="E51" t="s">
+        <v>233</v>
+      </c>
+      <c r="F51" t="s">
+        <v>199</v>
+      </c>
+      <c r="G51" t="s">
+        <v>183</v>
+      </c>
+      <c r="H51" t="s">
+        <v>183</v>
+      </c>
+      <c r="I51" t="s">
+        <v>274</v>
+      </c>
+      <c r="J51" t="s">
+        <v>237</v>
+      </c>
+      <c r="K51" t="s">
+        <v>191</v>
+      </c>
+      <c r="L51" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>